<commit_message>
Mystery no longer lingers
</commit_message>
<xml_diff>
--- a/Div_Roads Project.xlsx
+++ b/Div_Roads Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94b8e39c9d805aa/Documents/GitHub/Diverging-Roads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="256" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF4ADE64-D8E6-442A-9E93-175C62B43217}"/>
+  <xr:revisionPtr revIDLastSave="258" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FE6C09B-255E-41C4-AD32-F91F90CFC997}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18540" windowHeight="14505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="18540" windowHeight="14505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -947,6 +947,9 @@
       <c r="B12" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="C12" s="2">
+        <v>6216</v>
+      </c>
       <c r="D12" s="2">
         <v>2023</v>
       </c>
@@ -973,6 +976,9 @@
       <c r="B13" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="C13" s="2">
+        <v>934</v>
+      </c>
       <c r="D13" s="2">
         <v>2023</v>
       </c>
@@ -1220,7 +1226,7 @@
       </c>
       <c r="C32" s="2">
         <f>SUM(C2:C31)</f>
-        <v>21188</v>
+        <v>28338</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1229,7 +1235,7 @@
       </c>
       <c r="C33" s="10">
         <f>AVERAGE(C2:C31)</f>
-        <v>2118.8000000000002</v>
+        <v>2361.5</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fixed - Brilliant Mind
</commit_message>
<xml_diff>
--- a/Div_Roads Project.xlsx
+++ b/Div_Roads Project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94b8e39c9d805aa/Documents/GitHub/Diverging-Roads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="324" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D144B11-9C3A-4CB9-A5F4-66A43FEF6F42}"/>
+  <xr:revisionPtr revIDLastSave="334" documentId="11_F25DC773A252ABDACC10484719DA7CD85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA98F272-53E2-4C9E-A299-60A3A1DD0CF5}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16740" windowHeight="14505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="57">
   <si>
     <t>Title</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Copyright added</t>
   </si>
   <si>
-    <t>Text in original and lebtown differ - reconcile</t>
-  </si>
-  <si>
     <t>Done, defined the small and medium plate sizes in readme file.</t>
   </si>
   <si>
@@ -207,6 +204,9 @@
   </si>
   <si>
     <t>6b</t>
+  </si>
+  <si>
+    <t>Redoing</t>
   </si>
 </sst>
 </file>
@@ -265,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -296,6 +296,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,13 +633,13 @@
         <v>41</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="N1" s="6"/>
     </row>
@@ -701,7 +704,7 @@
         <v>40</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>33</v>
@@ -733,10 +736,10 @@
         <v>33</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>33</v>
@@ -834,7 +837,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>13</v>
@@ -1098,7 +1101,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2">
         <v>2482</v>
@@ -1260,7 +1263,7 @@
       <c r="G22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="11"/>
       <c r="J22" s="3" t="s">
         <v>33</v>
       </c>
@@ -1268,21 +1271,33 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="C23" s="2">
+        <v>1468</v>
+      </c>
       <c r="D23" s="2">
         <v>2025</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>42</v>
+      <c r="F23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1292,13 +1307,22 @@
       <c r="B24" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="C24" s="2">
+        <v>2039</v>
+      </c>
       <c r="D24" s="2">
         <v>2025</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>33</v>
       </c>
+      <c r="H24" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="J24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1385,7 +1409,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D31" s="2">
         <v>2026</v>
@@ -1393,35 +1417,35 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C33" s="2">
         <f>SUM(C2:C32)</f>
-        <v>65202</v>
+        <v>68709</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C34" s="10">
         <f>AVERAGE(C2:C32)</f>
-        <v>3104.8571428571427</v>
+        <v>2987.3478260869565</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>